<commit_message>
Obras: obra_id 3 a 28 na lista de controle, igual à aba Obras da planilha do painel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2E5Bx53QkBSuQwqWFPosz
</commit_message>
<xml_diff>
--- a/dados/controle/controle_obras_arcgis.xlsx
+++ b/dados/controle/controle_obras_arcgis.xlsx
@@ -480,7 +480,7 @@
   <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -498,14 +498,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fonte: Tabela 84 – Evolução dos domicílios em risco de inundação (documento a identificar). Texto das obras copiado da tabela.</t>
+          <t>Fonte: Tabela 84 – Evolução dos domicílios em risco de inundação (documento a identificar). Texto das obras copiado da tabela. O obra_id é o mesmo da aba "Obras" da planilha do painel (1 e 2 são os canais do Sanbra e da Mauricéa) e deve ir no campo obra da camada do ArcGIS.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Nº</t>
+          <t>obra_id</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -536,7 +536,7 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -952,7 +952,7 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
@@ -1030,7 +1030,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
@@ -1210,6 +1210,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr"/>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="D32" s="5" t="inlineStr">
         <is>

</xml_diff>